<commit_message>
Include first rectifier diode. Make minor change to first block to remove a non-US sourced part.
</commit_message>
<xml_diff>
--- a/docs/BOM/BOM_V1.xlsx
+++ b/docs/BOM/BOM_V1.xlsx
@@ -83,10 +83,10 @@
     <t>C2</t>
   </si>
   <si>
-    <t>GRM21BR61H475KE51L</t>
-  </si>
-  <si>
-    <t>4.7 µF, 1206, X5R ceramic capacitor</t>
+    <t>C0805C106K8PACTU</t>
+  </si>
+  <si>
+    <t>10 µF, 0805, X5R ceramic capacitor</t>
   </si>
   <si>
     <t>M1</t>

</xml_diff>

<commit_message>
Fix syntax issue in BOM.
</commit_message>
<xml_diff>
--- a/docs/BOM/BOM_V1.xlsx
+++ b/docs/BOM/BOM_V1.xlsx
@@ -83,10 +83,10 @@
     <t>C2</t>
   </si>
   <si>
-    <t>C0805C106K8PACTU</t>
-  </si>
-  <si>
-    <t>10 µF, 0805, X5R ceramic capacitor</t>
+    <t>C1210C106K5PACTU</t>
+  </si>
+  <si>
+    <t>10 µF, 1210, X5R ceramic capacitor</t>
   </si>
   <si>
     <t>M1</t>

</xml_diff>